<commit_message>
Specify red status LED part
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/hardware/GamepadPMOD/bom/GamepadPMOD_elecrow.xlsx
+++ b/hardware/GamepadPMOD/bom/GamepadPMOD_elecrow.xlsx
@@ -509,12 +509,22 @@
           <t>D1</t>
         </is>
       </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>APT1608SURCK</t>
+        </is>
+      </c>
       <c r="C5" s="0" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>LED</t>
+          <t>Red LED, 630 nm, 0603 (1608 metric)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com.au/en/products/detail/kingbright/APT1608SURCK/386438</t>
         </is>
       </c>
     </row>

</xml_diff>